<commit_message>
Consultas e rorteiro de validacao
</commit_message>
<xml_diff>
--- a/data/base_teste_systock.xlsx
+++ b/data/base_teste_systock.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andreson.vaz\Documents\ANDRESON GLIN\TESTE\teste1\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andreson.vaz\Documents\ANDRESON GLIN\TESTE\systock\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2CF640037F656DF8571788CCDCDB3BC434203F49" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FDD7A2-40C6-4D72-AEB5-2FB817C8B31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="venda" sheetId="1" r:id="rId1"/>
@@ -480,12 +480,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -500,7 +506,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -513,6 +519,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1178,31 +1189,31 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
+      <c r="A16" s="8">
         <v>15</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="11">
         <v>45708</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="8">
         <v>27</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="8">
         <v>43.4</v>
       </c>
-      <c r="G16" s="1">
-        <v>1</v>
-      </c>
-      <c r="H16" s="1">
-        <v>1</v>
-      </c>
-      <c r="I16" s="1" t="s">
+      <c r="G16" s="8">
+        <v>1</v>
+      </c>
+      <c r="H16" s="8">
+        <v>1</v>
+      </c>
+      <c r="I16" s="8" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3110,40 +3121,40 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
+      <c r="A9" s="9">
         <v>8</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="12">
         <v>45690</v>
       </c>
-      <c r="C9" s="1">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="C9" s="9">
+        <v>1</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="9">
         <v>8</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="9">
         <v>29</v>
       </c>
-      <c r="H9" s="1">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6">
+      <c r="H9" s="9">
+        <v>1</v>
+      </c>
+      <c r="I9" s="12">
         <v>45702</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="9">
         <v>24</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="9">
         <v>35.880000000000003</v>
       </c>
-      <c r="L9" s="1">
+      <c r="L9" s="9">
         <v>8</v>
       </c>
     </row>
@@ -3376,40 +3387,40 @@
       </c>
     </row>
     <row r="16" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
+      <c r="A16" s="8">
         <v>15</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="10">
         <v>45692</v>
       </c>
-      <c r="C16" s="1">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="C16" s="8">
+        <v>1</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="8">
         <v>15</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16" s="8">
         <v>45</v>
       </c>
-      <c r="H16" s="1">
-        <v>1</v>
-      </c>
-      <c r="I16" s="6">
+      <c r="H16" s="8">
+        <v>1</v>
+      </c>
+      <c r="I16" s="10">
         <v>45661</v>
       </c>
-      <c r="J16" s="1">
-        <v>1</v>
-      </c>
-      <c r="K16" s="1">
+      <c r="J16" s="8">
+        <v>1</v>
+      </c>
+      <c r="K16" s="8">
         <v>85.04</v>
       </c>
-      <c r="L16" s="1">
+      <c r="L16" s="8">
         <v>15</v>
       </c>
     </row>
@@ -5670,31 +5681,31 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="6">
+      <c r="A16" s="10">
         <v>45670</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="1">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="C16" s="8">
+        <v>1</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="8">
         <v>15</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16" s="8">
         <v>68</v>
       </c>
-      <c r="H16" s="1">
-        <v>1</v>
-      </c>
-      <c r="I16" s="1">
+      <c r="H16" s="8">
+        <v>1</v>
+      </c>
+      <c r="I16" s="8">
         <v>95.58</v>
       </c>
     </row>
@@ -6949,28 +6960,28 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>1</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="A5" s="9">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="9">
         <v>73</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="9">
         <v>89.67</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="9">
         <v>7.75</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="9">
         <v>226.5</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="9" t="s">
         <v>101</v>
       </c>
     </row>
@@ -7053,28 +7064,28 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>1</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="A9" s="9">
+        <v>1</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="9">
         <v>71</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="9">
         <v>140.57</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="9">
         <v>149.5</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="9">
         <v>95.28</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="9" t="s">
         <v>105</v>
       </c>
     </row>
@@ -7235,28 +7246,28 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
-        <v>1</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="8">
+        <v>1</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="8">
         <v>131</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="8">
         <v>101.15</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="8">
         <v>107.6</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16" s="8">
         <v>29.24</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="H16" s="8" t="s">
         <v>112</v>
       </c>
     </row>
@@ -8474,10 +8485,10 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="9" t="s">
         <v>126</v>
       </c>
     </row>
@@ -8522,10 +8533,10 @@
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="8" t="s">
         <v>135</v>
       </c>
     </row>

</xml_diff>